<commit_message>
Calibrate FDE plan for ML to GenAI progression
Amp-Thread-ID: https://ampcode.com/threads/T-01a08b9e-457f-76ce-8c80-58d58c7da0cd
Co-authored-by: Amp <amp@ampcode.com>
</commit_message>
<xml_diff>
--- a/docs/FDE-45-Day-Plan.xlsx
+++ b/docs/FDE-45-Day-Plan.xlsx
@@ -11,14 +11,18 @@
     <sheet name="45-Day Plan" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Phase Overview" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Technical Index" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="_Lists" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet name="GenAI Pre-work" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="After Day 45" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="_Lists" sheetId="7" state="hidden" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'45-Day Plan'!$A$4:$M$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'45-Day Plan'!$A$4:$N$49</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'45-Day Plan'!$1:$4</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'45-Day Plan'!$A$1:$M$49</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'45-Day Plan'!$A$1:$N$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Phase Overview'!$A$4:$F$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Technical Index'!$A$4:$E$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Technical Index'!$A$4:$E$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'GenAI Pre-work'!$A$4:$F$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'After Day 45'!$A$4:$D$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -164,7 +168,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -193,11 +197,40 @@
         <color rgb="00CBD6CF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD6CF"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00CBD6CF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD6CF"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00CBD6CF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -254,6 +287,11 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="14" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -356,9 +394,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FDE45DayPlan" displayName="FDE45DayPlan" ref="A4:M49" headerRowCount="1">
-  <autoFilter ref="A4:M49"/>
-  <tableColumns count="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FDE45DayPlan" displayName="FDE45DayPlan" ref="A4:N49" headerRowCount="1">
+  <autoFilter ref="A4:N49"/>
+  <tableColumns count="14">
     <tableColumn id="1" name="Day"/>
     <tableColumn id="2" name="Phase"/>
     <tableColumn id="3" name="Daily objective"/>
@@ -372,6 +410,7 @@
     <tableColumn id="11" name="Effort"/>
     <tableColumn id="12" name="Status"/>
     <tableColumn id="13" name="Learner notes / evidence links"/>
+    <tableColumn id="14" name="ML/DL → GenAI/FDE bridge"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1"/>
 </table>
@@ -667,7 +706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -681,14 +720,14 @@
     <row r="1" ht="38" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>FDE FIELD LAB — 45-DAY INTENSIVE</t>
+          <t>FDE FIELD LAB — CALIBRATED 45-DAY INTENSIVE</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>A practical learning and delivery tracker for one Support Operations Copilot capstone.</t>
+          <t>Support Operations Copilot · customer-first FDE delivery · calibrated for ML foundations and newer GenAI application skills.</t>
         </is>
       </c>
     </row>
@@ -705,6 +744,11 @@
           <t>In 45 days, build one well-understood capstone demonstrating discovery, deterministic full-stack delivery, evaluated AI, controlled LangGraph orchestration, hybrid retrieval, safe enterprise integration, production operation, and impact communication. This is a strong foundation and portfolio project—not a promise of complete field readiness.</t>
         </is>
       </c>
+      <c r="B5" s="22" t="n"/>
+      <c r="C5" s="22" t="n"/>
+      <c r="D5" s="22" t="n"/>
+      <c r="E5" s="22" t="n"/>
+      <c r="F5" s="23" t="n"/>
     </row>
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
@@ -719,6 +763,11 @@
           <t>Work 3–4 focused hours on six days, then use each seventh day as a gate/review day. Filter the 45-Day Plan by phase or status. Record your notes and evidence. If a gate fails, close the evidence gap before advancing merely because the calendar changed.</t>
         </is>
       </c>
+      <c r="B8" s="22" t="n"/>
+      <c r="C8" s="22" t="n"/>
+      <c r="D8" s="22" t="n"/>
+      <c r="E8" s="22" t="n"/>
+      <c r="F8" s="23" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
@@ -727,12 +776,17 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="82" customHeight="1">
+    <row r="11" ht="100" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Frontend: React + TypeScript. API/contracts: Python, FastAPI, Pydantic. Transactional data: PostgreSQL, SQLAlchemy, Alembic. Testing: pytest and Playwright. Agent orchestration: LangGraph only from Day 20. Retrieval: vector plus BM25/keyword comparison. Integration: typed tools, webhook, one read-only MCP capability. Delivery/operations: Docker, GitHub Actions, OpenTelemetry-compatible telemetry. These are lab choices, not the definition of an FDE.</t>
-        </is>
-      </c>
+          <t>Candidate stack: React/TypeScript or Streamlit for UI; Python, FastAPI, and Pydantic for contracts; PostgreSQL, SQLAlchemy, and Alembic for durable state; pytest and browser tests; provider-neutral model adapter with optional LangChain; LangGraph only from Day 20; pgvector/embedding and BM25 comparison; one read-only MCP capability; Docker, GitHub Actions, OpenTelemetry-compatible telemetry, and optional LangSmith. Day 6 records the final UI and stack choices in an ADR. Frameworks are replaceable tools, not FDE outcomes.</t>
+        </is>
+      </c>
+      <c r="B11" s="22" t="n"/>
+      <c r="C11" s="22" t="n"/>
+      <c r="D11" s="22" t="n"/>
+      <c r="E11" s="22" t="n"/>
+      <c r="F11" s="23" t="n"/>
     </row>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
@@ -747,6 +801,11 @@
           <t>Learn one concept and failure mode → explain it → design it against the Northstar workflow → build the smallest useful behavior → break a plausible wrong implementation → record evidence and the next decision.</t>
         </is>
       </c>
+      <c r="B15" s="22" t="n"/>
+      <c r="C15" s="22" t="n"/>
+      <c r="D15" s="22" t="n"/>
+      <c r="E15" s="22" t="n"/>
+      <c r="F15" s="23" t="n"/>
     </row>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -761,6 +820,11 @@
           <t>The dependency path is: customer outcome → deterministic product → evaluated model → durable graph → authorized retrieval → safe integration → production evidence → pilot and case study. Frameworks are introduced only when a scenario requirement justifies them.</t>
         </is>
       </c>
+      <c r="B18" s="22" t="n"/>
+      <c r="C18" s="22" t="n"/>
+      <c r="D18" s="22" t="n"/>
+      <c r="E18" s="22" t="n"/>
+      <c r="F18" s="23" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -809,25 +873,57 @@
         <v/>
       </c>
     </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>LEARNER CALIBRATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="68" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Working assumption: Python/ML concepts such as datasets, metrics, error analysis, and experiments are familiar; production LLM concepts are newer. The ML/DL bridge column identifies what transfers and what is genuinely new. Revise this assumption when actual evidence differs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="24" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>JUDGMENT APPLIED TO THE REVISED APPROACH</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="68" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Kept the GenAI orientation, ML/DL bridge, framework clarity, and optional extension topics. Preserved the Support Operations Copilot, discovery-first Day 1, provider-neutral boundaries, authorized retrieval, and required bounded multi-agent comparison. Streamlit, LangChain, LangSmith, FAISS, and hosted vector stores remain evidence-based alternatives—not automatic choices.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="16">
+    <mergeCell ref="A24:F24"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A11:F11"/>
     <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A28:F28"/>
     <mergeCell ref="A14:F14"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A27:F27"/>
     <mergeCell ref="A8:F8"/>
     <mergeCell ref="A17:F17"/>
     <mergeCell ref="A18:F18"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="A15:F15"/>
     <mergeCell ref="A7:F7"/>
+    <mergeCell ref="A25:F25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
-    <oddHeader>&amp;C&amp;B FDE Field Lab — 45-Day Intensive</oddHeader>
-    <oddFooter>&amp;LGenerated from the repository roadmap&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddHeader>&amp;C&amp;B FDE Field Lab — Calibrated 45-Day Intensive</oddHeader>
+    <oddFooter>&amp;LSupport Operations Copilot&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -843,7 +939,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M49"/>
+  <dimension ref="A1:N49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -859,19 +955,20 @@
     <col width="11" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="35" customWidth="1" min="13" max="13"/>
+    <col width="48" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="38" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>45-DAY DAILY PLAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="33" customHeight="1">
+          <t>CALIBRATED 45-DAY DAILY PLAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Filterable roadmap: purpose, technicality, build, integration, evidence, and company relevance for every day.</t>
+          <t>Support Operations Copilot: daily purpose, technicality, build, integration, evidence, company value, and ML/DL-to-GenAI bridge.</t>
         </is>
       </c>
     </row>
@@ -941,8 +1038,13 @@
           <t>Learner notes / evidence links</t>
         </is>
       </c>
-    </row>
-    <row r="5" ht="104" customHeight="1">
+      <c r="N4" s="8" t="inlineStr">
+        <is>
+          <t>ML/DL → GenAI/FDE bridge</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="112" customHeight="1">
       <c r="A5" s="9" t="n">
         <v>1</v>
       </c>
@@ -1001,8 +1103,13 @@
           <t>Complete — revised</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="104" customHeight="1">
+      <c r="N5" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: ML problem framing and hypotheses. NEW: customer workflow ownership, guarded business outcomes, and FDE accountability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="112" customHeight="1">
       <c r="A6" s="9" t="n">
         <v>2</v>
       </c>
@@ -1061,8 +1168,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="104" customHeight="1">
+      <c r="N6" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: experimental hypotheses. NEW: stakeholder evidence, source/confidence tracking, and non-leading discovery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="112" customHeight="1">
       <c r="A7" s="9" t="n">
         <v>3</v>
       </c>
@@ -1121,8 +1233,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="8" ht="104" customHeight="1">
+      <c r="N7" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: pipeline bottleneck analysis. NEW: human handoffs, queue time, rework, and operational risk mapping.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="112" customHeight="1">
       <c r="A8" s="9" t="n">
         <v>4</v>
       </c>
@@ -1181,8 +1298,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="9" ht="104" customHeight="1">
+      <c r="N8" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: metric thresholds and test sets. NEW: user stories, behavioral acceptance criteria, and explicit product non-goals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="112" customHeight="1">
       <c r="A9" s="9" t="n">
         <v>5</v>
       </c>
@@ -1241,8 +1363,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="10" ht="104" customHeight="1">
+      <c r="N9" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: statistics and metric design. NEW: business baselines paired with quality, safety, and adoption guardrails.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="112" customHeight="1">
       <c r="A10" s="9" t="n">
         <v>6</v>
       </c>
@@ -1263,12 +1390,12 @@
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>C4 context/container views; data flow; trust boundaries; synchronous vs asynchronous work; ADR format. Default stack proposed: React/TypeScript, FastAPI/Pydantic, PostgreSQL.</t>
+          <t>C4 context/container views; data flow; trust boundaries; synchronous vs asynchronous work; ADR. UI decision matrix: React/TypeScript vs Streamlit. Candidate backend: FastAPI/Pydantic/PostgreSQL.</t>
         </is>
       </c>
       <c r="F10" s="11" t="inlineStr">
         <is>
-          <t>Draw context and container diagrams; write ADR-001 selecting the smallest viable baseline stack.</t>
+          <t>Draw context/container diagrams and ADR-001. Select React for durable workflow UX or Streamlit for rapid pilot UX using customer requirements—not another repository.</t>
         </is>
       </c>
       <c r="G10" s="11" t="inlineStr">
@@ -1301,8 +1428,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="11" ht="104" customHeight="1">
+      <c r="N10" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: ML system/data-flow design. NEW: customer trust boundaries, ADRs, ownership, and UI trade-off decisions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="112" customHeight="1">
       <c r="A11" s="9" t="n">
         <v>7</v>
       </c>
@@ -1361,8 +1493,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="12" ht="104" customHeight="1">
+      <c r="N11" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: experiment review. NEW: customer/architecture gate communication and evidence-based scope correction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="112" customHeight="1">
       <c r="A12" s="9" t="n">
         <v>8</v>
       </c>
@@ -1421,8 +1558,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="13" ht="104" customHeight="1">
+      <c r="N12" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: Python typing and data models. NEW: business invariants and legal workflow state transitions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="112" customHeight="1">
       <c r="A13" s="9" t="n">
         <v>9</v>
       </c>
@@ -1481,8 +1623,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="14" ht="104" customHeight="1">
+      <c r="N13" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: serving endpoints. NEW: public API contracts, retry semantics, idempotency, and stable errors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="112" customHeight="1">
       <c r="A14" s="9" t="n">
         <v>10</v>
       </c>
@@ -1541,8 +1688,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="15" ht="104" customHeight="1">
+      <c r="N14" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: SQL and feature-store thinking. NEW: transactional truth, audit history, constraints, and query-driven indexes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="112" customHeight="1">
       <c r="A15" s="9" t="n">
         <v>11</v>
       </c>
@@ -1601,8 +1753,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="16" ht="104" customHeight="1">
+      <c r="N15" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: reproducible data pipelines. NEW: controlled migrations, transaction boundaries, and rollback evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="112" customHeight="1">
       <c r="A16" s="9" t="n">
         <v>12</v>
       </c>
@@ -1661,8 +1818,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="17" ht="104" customHeight="1">
+      <c r="N16" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: baseline/control methodology. NEW: deterministic product fallback before probabilistic AI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="112" customHeight="1">
       <c r="A17" s="9" t="n">
         <v>13</v>
       </c>
@@ -1721,8 +1883,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="18" ht="104" customHeight="1">
+      <c r="N17" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: experiment provenance. NEW: human accountability, immutable decisions, and concurrency-safe review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="112" customHeight="1">
       <c r="A18" s="9" t="n">
         <v>14</v>
       </c>
@@ -1743,12 +1910,12 @@
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>React + TypeScript; accessible forms; async UI states; typed API client; validation and error recovery.</t>
+          <t>Implement the UI selected by Day 6 ADR: default React + TypeScript for a durable support workflow; Streamlit remains a valid rapid-pilot alternative. Cover forms, async states, errors, accessibility, and typed API calls.</t>
         </is>
       </c>
       <c r="F18" s="11" t="inlineStr">
         <is>
-          <t>Create ticket intake, queue, recommendation review, evidence placeholder, and history views.</t>
+          <t>Build ticket intake, queue, recommendation review, evidence placeholder, and history views with the selected UI. Connect them to FastAPI and test the complete human workflow.</t>
         </is>
       </c>
       <c r="G18" s="11" t="inlineStr">
@@ -1781,8 +1948,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="19" ht="104" customHeight="1">
+      <c r="N18" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: dashboard/app exposure. NEW: operator workflow, accessibility, recoverable UI states, and adoption evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="112" customHeight="1">
       <c r="A19" s="9" t="n">
         <v>15</v>
       </c>
@@ -1841,8 +2013,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="20" ht="104" customHeight="1">
+      <c r="N19" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: model test discipline. NEW: browser-to-database release gate and deterministic product baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="112" customHeight="1">
       <c r="A20" s="9" t="n">
         <v>16</v>
       </c>
@@ -1863,12 +2040,12 @@
       </c>
       <c r="E20" s="11" t="inlineStr">
         <is>
-          <t>JSONL/CSV eval cases; independent labels; train/dev/test separation concept; precision, recall, F1, confusion matrix.</t>
+          <t>Independently labelled JSONL/CSV cases; category/priority/escalation labels; precision, recall, F1, confusion matrix; error slicing. Introduce LLM-as-judge limitations, but do not use RAGAS for classification.</t>
         </is>
       </c>
       <c r="F20" s="11" t="inlineStr">
         <is>
-          <t>Label representative ticket categories, priorities, risky actions, and expected escalation behavior; score deterministic rules.</t>
+          <t>Label representative ticket cases and score deterministic rules. Record expected route and approval behavior for later trace evaluation.</t>
         </is>
       </c>
       <c r="G20" s="11" t="inlineStr">
@@ -1901,8 +2078,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="21" ht="104" customHeight="1">
+      <c r="N20" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: labelled datasets, precision, recall, F1, and error slicing. NEW: agent trajectory fields and escalation labels.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="112" customHeight="1">
       <c r="A21" s="9" t="n">
         <v>17</v>
       </c>
@@ -1923,12 +2105,12 @@
       </c>
       <c r="E21" s="11" t="inlineStr">
         <is>
-          <t>Provider-neutral model interface; Pydantic structured output; JSON schema; timeout; parse/validation failure; test fake.</t>
+          <t>Provider-neutral model interface; Pydantic structured output/JSON Schema; invalid-output handling; timeout; test fake. LangChain may implement the adapter, but application contracts remain framework-independent.</t>
         </is>
       </c>
       <c r="F21" s="11" t="inlineStr">
         <is>
-          <t>Implement ticket classification behind an adapter; reject or repair invalid schema without silently accepting it.</t>
+          <t>Implement classification behind the adapter. If LangChain is used, contain it inside the adapter and test valid, malformed, missing-field, timeout, and provider-error responses.</t>
         </is>
       </c>
       <c r="G21" s="11" t="inlineStr">
@@ -1961,8 +2143,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="22" ht="104" customHeight="1">
+      <c r="N21" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: model-serving abstraction. NEW: untrusted LLM output, schema validation, parse failure, timeout, and provider fallback.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="112" customHeight="1">
       <c r="A22" s="9" t="n">
         <v>18</v>
       </c>
@@ -1983,12 +2170,12 @@
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>Prompt/config versioning; token counting; temperature control; model routing experiment; eval reproducibility.</t>
+          <t>Prompt/config versioning; token counting; sampling controls; small-versus-large model experiment; optional LangSmith experiment tracing; reproducible dataset/version linkage.</t>
         </is>
       </c>
       <c r="F22" s="11" t="inlineStr">
         <is>
-          <t>Evaluate a smaller/faster model and a larger reasoning model on the Day 16 dataset.</t>
+          <t>Compare a small fast model and a stronger reasoning model on Day 16 cases. Report quality, p50/p95 latency, tokens, cost, and failures without binding product logic to LangSmith.</t>
         </is>
       </c>
       <c r="G22" s="11" t="inlineStr">
@@ -2021,8 +2208,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="23" ht="104" customHeight="1">
+      <c r="N22" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: model comparison. NEW: prompts/config as versioned artifacts plus token, latency, and cost accounting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="112" customHeight="1">
       <c r="A23" s="9" t="n">
         <v>19</v>
       </c>
@@ -2081,8 +2273,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="24" ht="104" customHeight="1">
+      <c r="N23" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: ensemble/gating intuition. NEW: task-and-risk routing, budget enforcement, abstention, and deterministic fallback.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="112" customHeight="1">
       <c r="A24" s="9" t="n">
         <v>20</v>
       </c>
@@ -2103,12 +2300,12 @@
       </c>
       <c r="E24" s="11" t="inlineStr">
         <is>
-          <t>LangGraph StateGraph; TypedDict/Pydantic state; pure nodes; edges; reducers; ephemeral run state vs PostgreSQL business history.</t>
+          <t>LangGraph StateGraph; TypedDict/Pydantic state; nodes; edges; reducers; in-memory checkpoint only for learning. Separate ephemeral workflow state from PostgreSQL business history.</t>
         </is>
       </c>
       <c r="F24" s="11" t="inlineStr">
         <is>
-          <t>Model intake → validate → classify → route → prepare-review as minimal nodes and edges.</t>
+          <t>Model intake → validate → classify → route → prepare-review as minimal nodes and edges. Reuse existing domain services rather than moving business logic into graph nodes.</t>
         </is>
       </c>
       <c r="G24" s="11" t="inlineStr">
@@ -2141,8 +2338,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="25" ht="104" customHeight="1">
+      <c r="N24" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: computational graph intuition. NEW: LangGraph workflow state, nodes/edges, reducers, and separation from business history.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="112" customHeight="1">
       <c r="A25" s="9" t="n">
         <v>21</v>
       </c>
@@ -2163,12 +2365,12 @@
       </c>
       <c r="E25" s="11" t="inlineStr">
         <is>
-          <t>Conditional edges; stable run ID; LangGraph checkpointer; interrupt/resume; idempotent node design; correlation IDs.</t>
+          <t>Conditional edges; stable run ID; durable PostgreSQL-backed checkpointer; interrupt/resume; idempotent nodes; correlation IDs.</t>
         </is>
       </c>
       <c r="F25" s="11" t="inlineStr">
         <is>
-          <t>Pause before human review, persist checkpoint, simulate restart, then resume exactly once after a decision.</t>
+          <t>Pause before human review, persist the checkpoint, restart, and resume exactly once. Correlate graph run with the immutable business decision.</t>
         </is>
       </c>
       <c r="G25" s="11" t="inlineStr">
@@ -2201,8 +2403,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="26" ht="104" customHeight="1">
+      <c r="N25" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: checkpoint concepts. NEW: durable human interrupt/resume, stable run identity, and exactly-once effects.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="112" customHeight="1">
       <c r="A26" s="9" t="n">
         <v>22</v>
       </c>
@@ -2261,8 +2468,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="27" ht="104" customHeight="1">
+      <c r="N26" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: end-to-end evaluation. NEW: trace-level assertions for routes, calls, fallback, approval, and restart behavior.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="112" customHeight="1">
       <c r="A27" s="9" t="n">
         <v>23</v>
       </c>
@@ -2321,8 +2533,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="28" ht="104" customHeight="1">
+      <c r="N27" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: data ingestion. NEW: source lineage, parser quarantine, content trust, and document lifecycle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="112" customHeight="1">
       <c r="A28" s="9" t="n">
         <v>24</v>
       </c>
@@ -2381,8 +2598,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="29" ht="104" customHeight="1">
+      <c r="N28" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: preprocessing and sequence windows. NEW: semantic chunk boundaries, stable IDs, citation lineage, and incremental versions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="112" customHeight="1">
       <c r="A29" s="9" t="n">
         <v>25</v>
       </c>
@@ -2403,12 +2625,12 @@
       </c>
       <c r="E29" s="11" t="inlineStr">
         <is>
-          <t>Embeddings; vector dimensions; cosine similarity; pgvector/HNSW concepts; top-k; Recall@k.</t>
+          <t>Embedding model comparison; vector dimensions; cosine similarity; pgvector/HNSW concepts; optional local sentence-transformers/FAISS experiment; top-k; Recall@k.</t>
         </is>
       </c>
       <c r="F29" s="11" t="inlineStr">
         <is>
-          <t>Embed chunks, create a vector index, retrieve against labelled support questions, and record misses.</t>
+          <t>Embed stable chunks and build the authorization-capable candidate index in pgvector. Optionally compare local FAISS for learning; do not claim FAISS enforces tenant metadata.</t>
         </is>
       </c>
       <c r="G29" s="11" t="inlineStr">
@@ -2441,8 +2663,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="30" ht="104" customHeight="1">
+      <c r="N29" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: embeddings and similarity. NEW: retrieval Recall@k, index operations, context use, and tenant-safe candidates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="112" customHeight="1">
       <c r="A30" s="9" t="n">
         <v>26</v>
       </c>
@@ -2501,8 +2728,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="31" ht="104" customHeight="1">
+      <c r="N30" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: information-retrieval basics. NEW: BM25 as the exact-code complement to semantic search.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="112" customHeight="1">
       <c r="A31" s="9" t="n">
         <v>27</v>
       </c>
@@ -2561,8 +2793,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="32" ht="104" customHeight="1">
+      <c r="N31" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: ranking and reranking. NEW: reciprocal-rank fusion, context-token budgets, citations, and abstention.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="112" customHeight="1">
       <c r="A32" s="9" t="n">
         <v>28</v>
       </c>
@@ -2583,12 +2820,12 @@
       </c>
       <c r="E32" s="11" t="inlineStr">
         <is>
-          <t>Pre-filtered retrieval; tenant/ACL metadata; upsert; tombstone/delete; re-index queue; freshness lag; reconciliation.</t>
+          <t>Tenant/ACL filtering before scoring; authorized candidate set; upsert; tombstone/delete; re-index queue; freshness lag; reconciliation. Vector-store metadata filters are an optimization, not the authorization source.</t>
         </is>
       </c>
       <c r="F32" s="11" t="inlineStr">
         <is>
-          <t>Apply access filters before ranking; update one document; remove one; prove index/database convergence.</t>
+          <t>Apply authorization before vector and keyword ranking. Update one document, remove one, revoke one permission, and prove database/index convergence.</t>
         </is>
       </c>
       <c r="G32" s="11" t="inlineStr">
@@ -2621,8 +2858,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="33" ht="104" customHeight="1">
+      <c r="N32" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: dataset versioning. NEW: authorization before ranking, deletion propagation, freshness lag, and reconciliation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="112" customHeight="1">
       <c r="A33" s="9" t="n">
         <v>29</v>
       </c>
@@ -2643,12 +2885,12 @@
       </c>
       <c r="E33" s="11" t="inlineStr">
         <is>
-          <t>Recall@k; Precision@k; MRR/nDCG concepts; latency; index cost; error slicing.</t>
+          <t>Recall@k, Precision@k, MRR/nDCG, latency, cost, and query slicing. RAGAS/DeepEval or an LLM judge may supplement grounded-answer checks; independently labelled retrieval evidence remains primary.</t>
         </is>
       </c>
       <c r="F33" s="11" t="inlineStr">
         <is>
-          <t>Run the same labelled queries through all three strategies and document which query types each serves best.</t>
+          <t>Compare vector, keyword, and hybrid retrieval on identical queries. Add secondary grounded-answer evaluation and document judge disagreement or instability.</t>
         </is>
       </c>
       <c r="G33" s="11" t="inlineStr">
@@ -2681,8 +2923,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="34" ht="104" customHeight="1">
+      <c r="N33" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: benchmark comparison. NEW: select retrieval architecture from query slices, latency, cost, ACL, and citation evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="112" customHeight="1">
       <c r="A34" s="9" t="n">
         <v>30</v>
       </c>
@@ -2741,8 +2988,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="35" ht="104" customHeight="1">
+      <c r="N34" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: service authentication awareness. NEW: OIDC/JWT validation, RBAC, object ownership, tenancy, and audit policy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="112" customHeight="1">
       <c r="A35" s="9" t="n">
         <v>31</v>
       </c>
@@ -2801,8 +3053,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="36" ht="104" customHeight="1">
+      <c r="N35" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: adversarial ML mindset. NEW: direct/indirect prompt injection, content isolation, PII minimization, and exfiltration paths.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="112" customHeight="1">
       <c r="A36" s="9" t="n">
         <v>32</v>
       </c>
@@ -2861,8 +3118,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="37" ht="104" customHeight="1">
+      <c r="N36" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: callable model functions. NEW: tools as strict APIs with read/write separation, authorization, idempotency, and structured errors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="112" customHeight="1">
       <c r="A37" s="9" t="n">
         <v>33</v>
       </c>
@@ -2921,8 +3183,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="38" ht="104" customHeight="1">
+      <c r="N37" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: event pipelines. NEW: webhook signatures, replay windows, duplicate/out-of-order handling, and reconciliation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="112" customHeight="1">
       <c r="A38" s="9" t="n">
         <v>34</v>
       </c>
@@ -2981,8 +3248,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="39" ht="104" customHeight="1">
+      <c r="N38" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: human-in-the-loop review. NEW: approval over the exact immutable action, expiry, separation of duties, and compare-and-execute.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="112" customHeight="1">
       <c r="A39" s="9" t="n">
         <v>35</v>
       </c>
@@ -3041,8 +3313,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="40" ht="104" customHeight="1">
+      <c r="N39" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: model/tool interfaces. NEW: MCP host/client/server trust boundary and allowlisted read-only capability discovery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="112" customHeight="1">
       <c r="A40" s="9" t="n">
         <v>36</v>
       </c>
@@ -3101,8 +3378,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="41" ht="104" customHeight="1">
+      <c r="N40" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: adversarial testing. NEW: confused-deputy, cross-tenant, stale-approval, hostile-tool, and hostile-MCP scenarios.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="112" customHeight="1">
       <c r="A41" s="9" t="n">
         <v>37</v>
       </c>
@@ -3123,12 +3405,12 @@
       </c>
       <c r="E41" s="11" t="inlineStr">
         <is>
-          <t>OpenTelemetry concepts; structured logs; trace/span IDs; model/retrieval/tool/approval spans; token/cost metrics; PII redaction.</t>
+          <t>OpenTelemetry-compatible traces; structured logs; trace/span IDs; model/retrieval/tool/approval spans; token/cost metrics; PII redaction. LangSmith is an optional LLM trace view, not the only telemetry store.</t>
         </is>
       </c>
       <c r="F41" s="11" t="inlineStr">
         <is>
-          <t>Trace one ticket from HTTP request through graph, retrieval, model, tool proposal, approval, and result.</t>
+          <t>Trace one ticket end to end. If LangSmith is enabled, correlate it with the vendor-neutral run/trace ID and verify sensitive content is excluded.</t>
         </is>
       </c>
       <c r="G41" s="11" t="inlineStr">
@@ -3161,8 +3443,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="42" ht="104" customHeight="1">
+      <c r="N41" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: experiment tracking. NEW: production request traces spanning API, graph, retrieval, model, tools, approval, tokens, and cost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="112" customHeight="1">
       <c r="A42" s="9" t="n">
         <v>38</v>
       </c>
@@ -3221,8 +3508,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="43" ht="104" customHeight="1">
+      <c r="N42" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: resilient serving concepts. NEW: dependency-specific timeout/retry/fallback policies and uncertain-write handling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="112" customHeight="1">
       <c r="A43" s="9" t="n">
         <v>39</v>
       </c>
@@ -3281,8 +3573,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="44" ht="104" customHeight="1">
+      <c r="N43" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: batch/stream processing. NEW: at-least-once agent jobs, leases, dead letters, backpressure, and side-effect reconciliation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="112" customHeight="1">
       <c r="A44" s="9" t="n">
         <v>40</v>
       </c>
@@ -3303,12 +3600,12 @@
       </c>
       <c r="E44" s="11" t="inlineStr">
         <is>
-          <t>Docker/Compose; GitHub Actions; lint/type/test/security gates; migration job; staged environments; health/readiness; rollback.</t>
+          <t>Docker/Compose; GitHub Actions; lint/type/test/security/migration gates; staged deployment; health/readiness; rollback. Stable local/fake eval subset on PRs; full provider eval scheduled or manually approved.</t>
         </is>
       </c>
       <c r="F44" s="11" t="inlineStr">
         <is>
-          <t>Containerize services, run CI on a clean checkout, deploy to staging, migrate, smoke-test, and rehearse rollback.</t>
+          <t>Containerize services and run CI on a clean checkout. Block deterministic regressions on every PR; run costly/nondeterministic model evaluation under an explicit cadence and budget.</t>
         </is>
       </c>
       <c r="G44" s="11" t="inlineStr">
@@ -3341,8 +3638,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="45" ht="104" customHeight="1">
+      <c r="N44" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: MLOps pipelines. NEW: application migrations, staged delivery, rollback, deterministic PR gates, and scheduled full-model evals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="112" customHeight="1">
       <c r="A45" s="9" t="n">
         <v>41</v>
       </c>
@@ -3363,12 +3665,12 @@
       </c>
       <c r="E45" s="11" t="inlineStr">
         <is>
-          <t>SLI/SLO/error budget; Prometheus-compatible metrics concepts; dashboard; alert thresholds; load model; runbook; game day.</t>
+          <t>Availability, latency, and cost SLIs/SLOs; online quality proxies; offline labelled quality gate; dashboard; alerts; load model; runbook; game day. Do not describe unlabelled production RAGAS scores as a p95 truth metric.</t>
         </is>
       </c>
       <c r="F45" s="11" t="inlineStr">
         <is>
-          <t>Set availability/latency/quality targets, load representative traffic, inject one dependency failure, and follow the runbook.</t>
+          <t>Set service targets, evaluate quality offline, monitor abstention/rejection/citation proxies online, load test, inject one provider failure, and follow the runbook.</t>
         </is>
       </c>
       <c r="G45" s="11" t="inlineStr">
@@ -3401,8 +3703,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="46" ht="104" customHeight="1">
+      <c r="N45" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: model monitoring. NEW: service SLOs, online quality proxies, offline quality gates, alerts, runbooks, and game days.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="112" customHeight="1">
       <c r="A46" s="9" t="n">
         <v>42</v>
       </c>
@@ -3461,8 +3768,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="47" ht="104" customHeight="1">
+      <c r="N46" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: ensemble/specialist intuition. NEW: bounded multi-agent roles, typed handoffs, independent context, stop conditions, and added risks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="112" customHeight="1">
       <c r="A47" s="9" t="n">
         <v>43</v>
       </c>
@@ -3521,8 +3833,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="48" ht="104" customHeight="1">
+      <c r="N47" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: A/B evaluation. NEW: architecture decision from paired quality, latency, cost, token, and failure evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="112" customHeight="1">
       <c r="A48" s="9" t="n">
         <v>44</v>
       </c>
@@ -3581,8 +3898,13 @@
           <t>Not Started</t>
         </is>
       </c>
-    </row>
-    <row r="49" ht="104" customHeight="1">
+      <c r="N48" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: user-study thinking. NEW: rollout cohort, enablement, adoption funnel, support log, and prioritized field feedback.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="112" customHeight="1">
       <c r="A49" s="9" t="n">
         <v>45</v>
       </c>
@@ -3641,12 +3963,17 @@
           <t>Not Started</t>
         </is>
       </c>
+      <c r="N49" s="24" t="inlineStr">
+        <is>
+          <t>REUSES: model/report communication. NEW: guarded business-impact claim, architecture defense, customer narrative, and portfolio case study.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:M49"/>
+  <autoFilter ref="A4:N49"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
   </mergeCells>
   <conditionalFormatting sqref="L5:L49">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -3667,8 +3994,8 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;C&amp;B FDE Field Lab — 45-Day Intensive</oddHeader>
-    <oddFooter>&amp;LGenerated from the repository roadmap&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddHeader>&amp;C&amp;B FDE Field Lab — Calibrated 45-Day Intensive</oddHeader>
+    <oddFooter>&amp;LSupport Operations Copilot&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -3941,8 +4268,8 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
-    <oddHeader>&amp;C&amp;B FDE Field Lab — 45-Day Intensive</oddHeader>
-    <oddFooter>&amp;LGenerated from the repository roadmap&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddHeader>&amp;C&amp;B FDE Field Lab — Calibrated 45-Day Intensive</oddHeader>
+    <oddFooter>&amp;LSupport Operations Copilot&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -3958,7 +4285,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -3971,14 +4298,14 @@
     <row r="1" ht="38" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>TECHNICAL INDEX</t>
+          <t>FRAMEWORK &amp; TECHNICAL INDEX</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>When each major capability appears, where it becomes deeper, why it exists, and when not to use it.</t>
+          <t>What is core, conditional, or optional; when it appears; why it exists; and when not to use it.</t>
         </is>
       </c>
     </row>
@@ -4044,7 +4371,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>Day 6 decision; Day 14 build</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
@@ -4054,12 +4381,12 @@
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Accessible operator UI and typed browser/API boundary.</t>
+          <t>Default durable operator UI; compared with Streamlit against customer UX and timeline needs.</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>Do not build UI before core workflow and API contracts are clear.</t>
+          <t>Do not choose it merely to prove frontend breadth when a rapid pilot is the actual requirement.</t>
         </is>
       </c>
     </row>
@@ -4201,7 +4528,7 @@
     <row r="12" ht="63" customHeight="1">
       <c r="A12" s="21" t="inlineStr">
         <is>
-          <t>Model adapter / structured output</t>
+          <t>Provider-neutral model adapter</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
@@ -4216,12 +4543,12 @@
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Provider-neutral model calls with schema validation and fallback.</t>
+          <t>Stable application contract around model calls; LangChain may be contained as one implementation.</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>Do not trust free-form model text as an application contract.</t>
+          <t>Do not let provider or LangChain response objects become domain models.</t>
         </is>
       </c>
     </row>
@@ -4297,19 +4624,19 @@
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>Compare behavior against independent labels and regression thresholds.</t>
+          <t>Independent labels for task, route, trace, and retrieval regression evidence.</t>
         </is>
       </c>
       <c r="E15" s="11" t="inlineStr">
         <is>
-          <t>Do not select architecture from a few hand-picked demos.</t>
+          <t>Do not replace labels with an LLM judge or a few attractive examples.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="63" customHeight="1">
       <c r="A16" s="21" t="inlineStr">
         <is>
-          <t>Vector retrieval / pgvector</t>
+          <t>Embeddings + pgvector</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
@@ -4324,12 +4651,12 @@
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Semantic retrieval when query and source use different wording.</t>
+          <t>Semantic retrieval with transactional metadata and authorization-capable query paths; FAISS is an optional local comparison.</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
-          <t>Do not depend on it alone for exact identifiers or access control.</t>
+          <t>Do not depend on semantic similarity alone for exact identifiers or authorization.</t>
         </is>
       </c>
     </row>
@@ -4540,12 +4867,12 @@
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Correlated traces, metrics, sanitized logs, token use, cost, and audit.</t>
+          <t>Vendor-neutral application traces and metrics; LangSmith may add an LLM-focused inspection view.</t>
         </is>
       </c>
       <c r="E24" s="11" t="inlineStr">
         <is>
-          <t>Do not log raw prompts, secrets, or PII by default.</t>
+          <t>Do not make production debugging dependent on one vendor or log raw sensitive content.</t>
         </is>
       </c>
     </row>
@@ -4630,16 +4957,151 @@
         </is>
       </c>
     </row>
+    <row r="28" ht="66" customHeight="1">
+      <c r="A28" s="21" t="inlineStr">
+        <is>
+          <t>Streamlit (UI alternative)</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>6 / 14</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="D28" s="11" t="inlineStr">
+        <is>
+          <t>Fast pilot UI when customer workflow and timeline do not justify a richer frontend.</t>
+        </is>
+      </c>
+      <c r="E28" s="11" t="inlineStr">
+        <is>
+          <t>Do not call it automatically correct because a reference repository uses it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="66" customHeight="1">
+      <c r="A29" s="21" t="inlineStr">
+        <is>
+          <t>LangChain (adapter option)</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="C29" s="11" t="inlineStr">
+        <is>
+          <t>18–22, 32</t>
+        </is>
+      </c>
+      <c r="D29" s="11" t="inlineStr">
+        <is>
+          <t>Convenient provider/tool integrations contained behind our typed contracts.</t>
+        </is>
+      </c>
+      <c r="E29" s="11" t="inlineStr">
+        <is>
+          <t>Do not spread framework-specific objects across product, domain, and API layers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="66" customHeight="1">
+      <c r="A30" s="21" t="inlineStr">
+        <is>
+          <t>RAGAS / DeepEval (secondary)</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>27 / 29</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>40–41</t>
+        </is>
+      </c>
+      <c r="D30" s="11" t="inlineStr">
+        <is>
+          <t>Supplement labelled retrieval and grounded-answer evaluation with framework metrics.</t>
+        </is>
+      </c>
+      <c r="E30" s="11" t="inlineStr">
+        <is>
+          <t>Do not use RAG metrics for classification or treat model-judge scores as ground truth.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="66" customHeight="1">
+      <c r="A31" s="21" t="inlineStr">
+        <is>
+          <t>LangSmith (optional)</t>
+        </is>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>16 / 18</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>22, 37–41</t>
+        </is>
+      </c>
+      <c r="D31" s="11" t="inlineStr">
+        <is>
+          <t>Experiment and LLM-trace inspection correlated with vendor-neutral run IDs.</t>
+        </is>
+      </c>
+      <c r="E31" s="11" t="inlineStr">
+        <is>
+          <t>Do not make it the sole source of business audit or operational telemetry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="66" customHeight="1">
+      <c r="A32" s="21" t="inlineStr">
+        <is>
+          <t>sentence-transformers / FAISS (comparison)</t>
+        </is>
+      </c>
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="D32" s="11" t="inlineStr">
+        <is>
+          <t>Local embedding and vector-search learning baseline.</t>
+        </is>
+      </c>
+      <c r="E32" s="11" t="inlineStr">
+        <is>
+          <t>Do not claim FAISS natively enforces tenant ACL metadata or durable lifecycle guarantees.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:E27"/>
+  <autoFilter ref="A4:E32"/>
   <mergeCells count="2">
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
-    <oddHeader>&amp;C&amp;B FDE Field Lab — 45-Day Intensive</oddHeader>
-    <oddFooter>&amp;LGenerated from the repository roadmap&amp;RPage &amp;P of &amp;N</oddFooter>
+    <oddHeader>&amp;C&amp;B FDE Field Lab — Calibrated 45-Day Intensive</oddHeader>
+    <oddFooter>&amp;LSupport Operations Copilot&amp;RPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -4651,6 +5113,450 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="0072D6B2"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="38" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>OPTIONAL GENAI PRE-WORK</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Complete between Days 1 and 2 if LLM application basics are unfamiliar. Total: approximately three hours.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Module</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Learn</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Hands-on exercise</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>Why it matters later</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="82" customHeight="1">
+      <c r="A5" s="21" t="inlineStr">
+        <is>
+          <t>1. Request anatomy</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="inlineStr">
+        <is>
+          <t>35 min</t>
+        </is>
+      </c>
+      <c r="C5" s="20" t="inlineStr">
+        <is>
+          <t>Provider API, system/user messages, model name, temperature, max output tokens.</t>
+        </is>
+      </c>
+      <c r="D5" s="20" t="inlineStr">
+        <is>
+          <t>Make one model call through a tiny provider-neutral function; inspect the raw response without exposing secrets.</t>
+        </is>
+      </c>
+      <c r="E5" s="20" t="inlineStr">
+        <is>
+          <t>Notebook/script plus redacted request/response anatomy.</t>
+        </is>
+      </c>
+      <c r="F5" s="20" t="inlineStr">
+        <is>
+          <t>Prevents later abstractions from hiding what the upstream dependency actually returns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="82" customHeight="1">
+      <c r="A6" s="21" t="inlineStr">
+        <is>
+          <t>2. Tokens, context, and cost</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="inlineStr">
+        <is>
+          <t>40 min</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>Tokenization, context window, input/output limits, truncation, and cost calculation.</t>
+        </is>
+      </c>
+      <c r="D6" s="20" t="inlineStr">
+        <is>
+          <t>Count tokens for short and long prompts; calculate cost for 1,000 requests; trigger a context-budget decision.</t>
+        </is>
+      </c>
+      <c r="E6" s="20" t="inlineStr">
+        <is>
+          <t>Token and cost table with assumptions.</t>
+        </is>
+      </c>
+      <c r="F6" s="20" t="inlineStr">
+        <is>
+          <t>Supports routing, retrieval context budgets, latency, and production cost controls.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="82" customHeight="1">
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>3. Variability and sampling</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="inlineStr">
+        <is>
+          <t>30 min</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>Probabilistic outputs, temperature, deterministic-seeming behavior, and seed limitations.</t>
+        </is>
+      </c>
+      <c r="D7" s="20" t="inlineStr">
+        <is>
+          <t>Run the same task repeatedly at two temperatures and categorize differences.</t>
+        </is>
+      </c>
+      <c r="E7" s="20" t="inlineStr">
+        <is>
+          <t>Small variability table and one failure observation.</t>
+        </is>
+      </c>
+      <c r="F7" s="20" t="inlineStr">
+        <is>
+          <t>Explains why ordinary unit tests alone cannot evaluate models.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="82" customHeight="1">
+      <c r="A8" s="21" t="inlineStr">
+        <is>
+          <t>4. Structured output</t>
+        </is>
+      </c>
+      <c r="B8" s="20" t="inlineStr">
+        <is>
+          <t>45 min</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>JSON Schema/Pydantic contract, parse failure, missing fields, and validation.</t>
+        </is>
+      </c>
+      <c r="D8" s="20" t="inlineStr">
+        <is>
+          <t>Request a small classification object; validate it; deliberately feed malformed output.</t>
+        </is>
+      </c>
+      <c r="E8" s="20" t="inlineStr">
+        <is>
+          <t>Passing and failing validation examples.</t>
+        </is>
+      </c>
+      <c r="F8" s="20" t="inlineStr">
+        <is>
+          <t>Prepares for Day 17 without accepting model text as trusted data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="82" customHeight="1">
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>5. Reliability and safety</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="inlineStr">
+        <is>
+          <t>30 min</t>
+        </is>
+      </c>
+      <c r="C9" s="20" t="inlineStr">
+        <is>
+          <t>Timeout, 429/5xx, secret handling, untrusted user content, and human escalation.</t>
+        </is>
+      </c>
+      <c r="D9" s="20" t="inlineStr">
+        <is>
+          <t>Use a fake client to simulate timeout and invalid output; return a safe machine-readable failure.</t>
+        </is>
+      </c>
+      <c r="E9" s="20" t="inlineStr">
+        <is>
+          <t>Two failure tests and no secret in source/logs.</t>
+        </is>
+      </c>
+      <c r="F9" s="20" t="inlineStr">
+        <is>
+          <t>Introduces the model as an unreliable dependency, not an autonomous authority.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:F9"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;B FDE Field Lab — Calibrated 45-Day Intensive</oddHeader>
+    <oddFooter>&amp;LSupport Operations Copilot&amp;RPage &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="0072D6B2"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="65" customWidth="1" min="2" max="2"/>
+    <col width="57" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="38" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>OPTIONAL DEPTH AFTER DAY 45</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>The intensive creates one strong capstone foundation. Choose follow-on depth from evidence and role requirements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Track</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Learn / build next</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Choose it when</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Do not choose it merely because…</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="72" customHeight="1">
+      <c r="A5" s="21" t="inlineStr">
+        <is>
+          <t>Advanced multi-agent</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="inlineStr">
+        <is>
+          <t>Supervisor/worker patterns, isolated memory, inter-agent failure recovery, and larger paired evaluations.</t>
+        </is>
+      </c>
+      <c r="C5" s="20" t="inlineStr">
+        <is>
+          <t>Day 42–43 shows measured role-separation value and the target role needs it.</t>
+        </is>
+      </c>
+      <c r="D5" s="20" t="inlineStr">
+        <is>
+          <t>Multiple agents look more advanced.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="72" customHeight="1">
+      <c r="A6" s="21" t="inlineStr">
+        <is>
+          <t>Fine-tuning and model customization</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="inlineStr">
+        <is>
+          <t>Dataset curation, LoRA/QLoRA concepts, serving, evaluation, drift, and rollback.</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>Prompting/retrieval cannot meet a measured task requirement and sufficient labelled data exists.</t>
+        </is>
+      </c>
+      <c r="D6" s="20" t="inlineStr">
+        <is>
+          <t>You already have ML/DL experience.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="72" customHeight="1">
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>Distributed production scale</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="inlineStr">
+        <is>
+          <t>Multi-region, data residency, distributed caches/queues, capacity, and disaster recovery.</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>A target customer or load model requires those constraints.</t>
+        </is>
+      </c>
+      <c r="D7" s="20" t="inlineStr">
+        <is>
+          <t>Kubernetes or microservices are common interview words.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="72" customHeight="1">
+      <c r="A8" s="21" t="inlineStr">
+        <is>
+          <t>Security and compliance</t>
+        </is>
+      </c>
+      <c r="B8" s="20" t="inlineStr">
+        <is>
+          <t>SOC 2/ISO control mapping, privacy impact assessment, red teaming, retention, and evidence packs.</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>The target industry, customer, or role has regulated-data obligations.</t>
+        </is>
+      </c>
+      <c r="D8" s="20" t="inlineStr">
+        <is>
+          <t>Security can be solved by adding more prompt instructions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="72" customHeight="1">
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>Cost and observability depth</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="inlineStr">
+        <is>
+          <t>Caching, provider negotiation, trace sampling, budget attribution, and quality/cost optimization.</t>
+        </is>
+      </c>
+      <c r="C9" s="20" t="inlineStr">
+        <is>
+          <t>Measured traffic or spend identifies a real optimization opportunity.</t>
+        </is>
+      </c>
+      <c r="D9" s="20" t="inlineStr">
+        <is>
+          <t>Premature optimization feels production-ready.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="72" customHeight="1">
+      <c r="A10" s="21" t="inlineStr">
+        <is>
+          <t>Second domain transfer</t>
+        </is>
+      </c>
+      <c r="B10" s="20" t="inlineStr">
+        <is>
+          <t>Apply the same FDE loop to incident response, contracts, or data operations.</t>
+        </is>
+      </c>
+      <c r="C10" s="20" t="inlineStr">
+        <is>
+          <t>You need evidence that the architecture and discovery skills transfer beyond support.</t>
+        </is>
+      </c>
+      <c r="D10" s="20" t="inlineStr">
+        <is>
+          <t>One capstone should become several shallow demos.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:D10"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;B FDE Field Lab — Calibrated 45-Day Intensive</oddHeader>
+    <oddFooter>&amp;LSupport Operations Copilot&amp;RPage &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>

</xml_diff>